<commit_message>
adds new reaches data
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_surveyed_reaches_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_surveyed_reaches_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063A6C99-3274-4668-9E4C-98FF1D107C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4545AD-6D14-4E1D-B9DF-2A22EEA15F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5310" yWindow="1150" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4050" yWindow="930" windowWidth="19200" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -100,13 +100,13 @@
     <t>surveyed_reaches</t>
   </si>
   <si>
-    <t>04/21/2003</t>
-  </si>
-  <si>
     <t>10/25/2024</t>
   </si>
   <si>
     <t>Reach surveyed for redds. Levels =c("R1", "R3", "R2", "R4", "R5", "R6", "R7", "R5A", "R5B", "R5C", "R6A", "R6B")</t>
+  </si>
+  <si>
+    <t>05/06/1995</t>
   </si>
 </sst>
 </file>
@@ -538,10 +538,10 @@
       </c>
       <c r="K2" s="14"/>
       <c r="L2" s="16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M2" s="16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -562,7 +562,7 @@
         <v>21</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>13</v>

</xml_diff>